<commit_message>
output: presupuestos_asesores_mayo_v2 - minimos corregidos
</commit_message>
<xml_diff>
--- a/docs/outputs/presupuestos_asesores_mayo.xlsx
+++ b/docs/outputs/presupuestos_asesores_mayo.xlsx
@@ -543,13 +543,13 @@
         <v>8411764</v>
       </c>
       <c r="N2" t="n">
-        <v>48310930</v>
+        <v>36378712</v>
       </c>
       <c r="O2" t="n">
-        <v>3090112</v>
+        <v>5000000</v>
       </c>
       <c r="P2" t="n">
-        <v>33474491</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="3">
@@ -597,13 +597,13 @@
         <v>7776470</v>
       </c>
       <c r="N3" t="n">
-        <v>4138377</v>
+        <v>10000000</v>
       </c>
       <c r="O3" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P3" t="n">
-        <v>8229509</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="4">
@@ -651,13 +651,13 @@
         <v>23529411</v>
       </c>
       <c r="N4" t="n">
-        <v>3167976</v>
+        <v>10000000</v>
       </c>
       <c r="O4" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P4" t="n">
-        <v>19631710</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="5">
@@ -705,13 +705,13 @@
         <v>22263865</v>
       </c>
       <c r="N5" t="n">
-        <v>31783096</v>
+        <v>23933054</v>
       </c>
       <c r="O5" t="n">
-        <v>2767598</v>
+        <v>5000000</v>
       </c>
       <c r="P5" t="n">
-        <v>28450448</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="6">
@@ -759,13 +759,13 @@
         <v>5642016</v>
       </c>
       <c r="N6" t="n">
-        <v>160616951</v>
+        <v>120946499</v>
       </c>
       <c r="O6" t="n">
-        <v>17008072</v>
+        <v>12807283</v>
       </c>
       <c r="P6" t="n">
-        <v>11038896</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="7">
@@ -813,13 +813,13 @@
         <v>4967226</v>
       </c>
       <c r="N7" t="n">
-        <v>58758236</v>
+        <v>44245659</v>
       </c>
       <c r="O7" t="n">
-        <v>5473444</v>
+        <v>5000000</v>
       </c>
       <c r="P7" t="n">
-        <v>14117627</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="8">
@@ -867,13 +867,13 @@
         <v>10627731</v>
       </c>
       <c r="N8" t="n">
-        <v>7405926</v>
+        <v>10000000</v>
       </c>
       <c r="O8" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P8" t="n">
-        <v>14204765</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="9">
@@ -921,13 +921,13 @@
         <v>14064705</v>
       </c>
       <c r="N9" t="n">
-        <v>70812905</v>
+        <v>53322970</v>
       </c>
       <c r="O9" t="n">
-        <v>3178274</v>
+        <v>5000000</v>
       </c>
       <c r="P9" t="n">
-        <v>18734845</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="10">
@@ -975,13 +975,13 @@
         <v>17435294</v>
       </c>
       <c r="N10" t="n">
-        <v>19687881</v>
+        <v>14825211</v>
       </c>
       <c r="O10" t="n">
-        <v>697481</v>
+        <v>5000000</v>
       </c>
       <c r="P10" t="n">
-        <v>38657634</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="11">
@@ -1029,13 +1029,13 @@
         <v>41681546</v>
       </c>
       <c r="N11" t="n">
-        <v>82846668</v>
+        <v>62384539</v>
       </c>
       <c r="O11" t="n">
-        <v>7798747</v>
+        <v>5872550</v>
       </c>
       <c r="P11" t="n">
-        <v>59977257</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="12">
@@ -1083,13 +1083,13 @@
         <v>43616806</v>
       </c>
       <c r="N12" t="n">
-        <v>101455109</v>
+        <v>76396919</v>
       </c>
       <c r="O12" t="n">
-        <v>5598433</v>
+        <v>5000000</v>
       </c>
       <c r="P12" t="n">
-        <v>61325107</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="13">
@@ -1137,13 +1137,13 @@
         <v>14152100</v>
       </c>
       <c r="N13" t="n">
-        <v>41518415</v>
+        <v>31263866</v>
       </c>
       <c r="O13" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P13" t="n">
-        <v>19523610</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="14">
@@ -1197,7 +1197,7 @@
         <v>5000000</v>
       </c>
       <c r="P14" t="n">
-        <v>13001401</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="15">
@@ -1245,13 +1245,13 @@
         <v>9329411</v>
       </c>
       <c r="N15" t="n">
-        <v>2982914</v>
+        <v>10000000</v>
       </c>
       <c r="O15" t="n">
         <v>5000000</v>
       </c>
       <c r="P15" t="n">
-        <v>13658292</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="16">
@@ -1299,13 +1299,13 @@
         <v>9771428</v>
       </c>
       <c r="N16" t="n">
-        <v>3855743</v>
+        <v>10000000</v>
       </c>
       <c r="O16" t="n">
         <v>5000000</v>
       </c>
       <c r="P16" t="n">
-        <v>10269468</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="17">
@@ -1359,7 +1359,7 @@
         <v>5000000</v>
       </c>
       <c r="P17" t="n">
-        <v>22944314</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="18">
@@ -1407,13 +1407,13 @@
         <v>15894117</v>
       </c>
       <c r="N18" t="n">
-        <v>8380012</v>
+        <v>10000000</v>
       </c>
       <c r="O18" t="n">
         <v>5000000</v>
       </c>
       <c r="P18" t="n">
-        <v>23027421</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="19">
@@ -1467,7 +1467,7 @@
         <v>5000000</v>
       </c>
       <c r="P19" t="n">
-        <v>14364706</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="20">
@@ -1521,7 +1521,7 @@
         <v>5000000</v>
       </c>
       <c r="P20" t="n">
-        <v>29705323</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="21">
@@ -1572,10 +1572,10 @@
         <v>11131093</v>
       </c>
       <c r="O21" t="n">
-        <v>271989</v>
+        <v>5000000</v>
       </c>
       <c r="P21" t="n">
-        <v>1410045</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="22">
@@ -1623,13 +1623,13 @@
         <v>28138655</v>
       </c>
       <c r="N22" t="n">
-        <v>7056023</v>
+        <v>10000000</v>
       </c>
       <c r="O22" t="n">
         <v>5000000</v>
       </c>
       <c r="P22" t="n">
-        <v>24211765</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="23">
@@ -1677,13 +1677,13 @@
         <v>14498319</v>
       </c>
       <c r="N23" t="n">
-        <v>3654062</v>
+        <v>10000000</v>
       </c>
       <c r="O23" t="n">
         <v>5000000</v>
       </c>
       <c r="P23" t="n">
-        <v>25435015</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="24">
@@ -1731,13 +1731,13 @@
         <v>6125974</v>
       </c>
       <c r="N24" t="n">
-        <v>981793</v>
+        <v>10000000</v>
       </c>
       <c r="O24" t="n">
         <v>5000000</v>
       </c>
       <c r="P24" t="n">
-        <v>2907538</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="25">
@@ -1785,13 +1785,13 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>4602522</v>
+        <v>10000000</v>
       </c>
       <c r="O25" t="n">
         <v>8461132</v>
       </c>
       <c r="P25" t="n">
-        <v>470309</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="26">
@@ -1842,10 +1842,10 @@
         <v>32232561</v>
       </c>
       <c r="O26" t="n">
-        <v>266334</v>
+        <v>5000000</v>
       </c>
       <c r="P26" t="n">
-        <v>16629922</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="27">
@@ -1896,10 +1896,10 @@
         <v>14958264</v>
       </c>
       <c r="O27" t="n">
-        <v>504202</v>
+        <v>5000000</v>
       </c>
       <c r="P27" t="n">
-        <v>24203244</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="28">
@@ -1947,13 +1947,13 @@
         <v>10415168</v>
       </c>
       <c r="N28" t="n">
-        <v>7538233</v>
+        <v>10000000</v>
       </c>
       <c r="O28" t="n">
-        <v>435295</v>
+        <v>5000000</v>
       </c>
       <c r="P28" t="n">
-        <v>12497213</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="29">
@@ -2001,7 +2001,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>7890163</v>
+        <v>10000000</v>
       </c>
       <c r="O29" t="n">
         <v>7015687</v>
@@ -2055,13 +2055,13 @@
         <v>9221008</v>
       </c>
       <c r="N30" t="n">
-        <v>9307003</v>
+        <v>10000000</v>
       </c>
       <c r="O30" t="n">
-        <v>2891059</v>
+        <v>5000000</v>
       </c>
       <c r="P30" t="n">
-        <v>15306163</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="31">
@@ -2115,7 +2115,7 @@
         <v>18482606</v>
       </c>
       <c r="P31" t="n">
-        <v>3925211</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="32">
@@ -2166,10 +2166,10 @@
         <v>42966359</v>
       </c>
       <c r="O32" t="n">
-        <v>846779</v>
+        <v>5000000</v>
       </c>
       <c r="P32" t="n">
-        <v>19699160</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="33">
@@ -2223,7 +2223,7 @@
         <v>8631491</v>
       </c>
       <c r="P33" t="n">
-        <v>2651541</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="34">
@@ -2274,10 +2274,10 @@
         <v>31217311</v>
       </c>
       <c r="O34" t="n">
-        <v>480953</v>
+        <v>5000000</v>
       </c>
       <c r="P34" t="n">
-        <v>19690757</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="35">
@@ -2331,7 +2331,7 @@
         <v>5000000</v>
       </c>
       <c r="P35" t="n">
-        <v>15865538</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="36">
@@ -2385,7 +2385,7 @@
         <v>21088740</v>
       </c>
       <c r="P36" t="n">
-        <v>1789636</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="37">
@@ -2439,7 +2439,7 @@
         <v>5000000</v>
       </c>
       <c r="P37" t="n">
-        <v>18621202</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="38">
@@ -2490,10 +2490,10 @@
         <v>55264524</v>
       </c>
       <c r="O38" t="n">
-        <v>374230</v>
+        <v>5000000</v>
       </c>
       <c r="P38" t="n">
-        <v>25875339</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="39">
@@ -2541,13 +2541,13 @@
         <v>16666386</v>
       </c>
       <c r="N39" t="n">
-        <v>8791597</v>
+        <v>10000000</v>
       </c>
       <c r="O39" t="n">
         <v>5000000</v>
       </c>
       <c r="P39" t="n">
-        <v>16977031</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="40">
@@ -2601,7 +2601,7 @@
         <v>5000000</v>
       </c>
       <c r="P40" t="n">
-        <v>24900169</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="41">
@@ -2652,10 +2652,10 @@
         <v>55949580</v>
       </c>
       <c r="O41" t="n">
-        <v>4806390</v>
+        <v>5000000</v>
       </c>
       <c r="P41" t="n">
-        <v>12549692</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="42">
@@ -2703,13 +2703,13 @@
         <v>4010924</v>
       </c>
       <c r="N42" t="n">
-        <v>5073307</v>
+        <v>10000000</v>
       </c>
       <c r="O42" t="n">
-        <v>6195001</v>
+        <v>5000000</v>
       </c>
       <c r="P42" t="n">
-        <v>1656513</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="43">
@@ -2757,13 +2757,13 @@
         <v>8773109</v>
       </c>
       <c r="N43" t="n">
-        <v>4061631</v>
+        <v>10000000</v>
       </c>
       <c r="O43" t="n">
-        <v>2658819</v>
+        <v>5000000</v>
       </c>
       <c r="P43" t="n">
-        <v>16424907</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="44">
@@ -2811,13 +2811,13 @@
         <v>6868907</v>
       </c>
       <c r="N44" t="n">
-        <v>34726012</v>
+        <v>28027451</v>
       </c>
       <c r="O44" t="n">
-        <v>12586437</v>
+        <v>10158544</v>
       </c>
       <c r="P44" t="n">
-        <v>5629642</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="45">
@@ -2865,13 +2865,13 @@
         <v>20982352</v>
       </c>
       <c r="N45" t="n">
-        <v>30799043</v>
+        <v>24857984</v>
       </c>
       <c r="O45" t="n">
-        <v>4248348</v>
+        <v>5000000</v>
       </c>
       <c r="P45" t="n">
-        <v>21464201</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="46">
@@ -2919,13 +2919,13 @@
         <v>5103361</v>
       </c>
       <c r="N46" t="n">
-        <v>11638272</v>
+        <v>10000000</v>
       </c>
       <c r="O46" t="n">
-        <v>3292896</v>
+        <v>5000000</v>
       </c>
       <c r="P46" t="n">
-        <v>12448654</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="47">
@@ -2973,13 +2973,13 @@
         <v>24199999</v>
       </c>
       <c r="N47" t="n">
-        <v>21658422</v>
+        <v>17480566</v>
       </c>
       <c r="O47" t="n">
-        <v>6195001</v>
+        <v>5000000</v>
       </c>
       <c r="P47" t="n">
-        <v>35284905</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="48">
@@ -3027,13 +3027,13 @@
         <v>30847731</v>
       </c>
       <c r="N48" t="n">
-        <v>66983961</v>
+        <v>54062922</v>
       </c>
       <c r="O48" t="n">
-        <v>18546470</v>
+        <v>14968902</v>
       </c>
       <c r="P48" t="n">
-        <v>31844516</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="49">
@@ -3081,13 +3081,13 @@
         <v>7328571</v>
       </c>
       <c r="N49" t="n">
-        <v>49327471</v>
+        <v>39812325</v>
       </c>
       <c r="O49" t="n">
-        <v>2167036</v>
+        <v>5000000</v>
       </c>
       <c r="P49" t="n">
-        <v>6525054</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="50">
@@ -3135,13 +3135,13 @@
         <v>6914285</v>
       </c>
       <c r="N50" t="n">
-        <v>1272665</v>
+        <v>10000000</v>
       </c>
       <c r="O50" t="n">
-        <v>6195001</v>
+        <v>5000000</v>
       </c>
       <c r="P50" t="n">
-        <v>2855601</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="51">
@@ -3189,13 +3189,13 @@
         <v>25538655</v>
       </c>
       <c r="N51" t="n">
-        <v>59300554</v>
+        <v>47861625</v>
       </c>
       <c r="O51" t="n">
-        <v>12201098</v>
+        <v>9847536</v>
       </c>
       <c r="P51" t="n">
-        <v>24953356</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="52">
@@ -3243,13 +3243,13 @@
         <v>2079831</v>
       </c>
       <c r="N52" t="n">
-        <v>9061707</v>
+        <v>10000000</v>
       </c>
       <c r="O52" t="n">
-        <v>6195001</v>
+        <v>5000000</v>
       </c>
       <c r="P52" t="n">
-        <v>4684948</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="53">
@@ -3297,13 +3297,13 @@
         <v>16697478</v>
       </c>
       <c r="N53" t="n">
-        <v>53925654</v>
+        <v>43523530</v>
       </c>
       <c r="O53" t="n">
-        <v>8733042</v>
+        <v>7048460</v>
       </c>
       <c r="P53" t="n">
-        <v>12479542</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="54">
@@ -3351,13 +3351,13 @@
         <v>14551680</v>
       </c>
       <c r="N54" t="n">
-        <v>6192541</v>
+        <v>10000000</v>
       </c>
       <c r="O54" t="n">
-        <v>539331</v>
+        <v>5000000</v>
       </c>
       <c r="P54" t="n">
-        <v>18329993</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="55">
@@ -3405,13 +3405,13 @@
         <v>20524033</v>
       </c>
       <c r="N55" t="n">
-        <v>95839708</v>
+        <v>77352468</v>
       </c>
       <c r="O55" t="n">
-        <v>6235954</v>
+        <v>5033054</v>
       </c>
       <c r="P55" t="n">
-        <v>29598869</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="56">
@@ -3459,13 +3459,13 @@
         <v>31865546</v>
       </c>
       <c r="N56" t="n">
-        <v>4861037</v>
+        <v>10000000</v>
       </c>
       <c r="O56" t="n">
         <v>5000000</v>
       </c>
       <c r="P56" t="n">
-        <v>29066387</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="57">
@@ -3516,10 +3516,10 @@
         <v>15572269</v>
       </c>
       <c r="O57" t="n">
-        <v>4063586</v>
+        <v>5000000</v>
       </c>
       <c r="P57" t="n">
-        <v>18670393</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="58">
@@ -3567,13 +3567,13 @@
         <v>12105042</v>
       </c>
       <c r="N58" t="n">
-        <v>5640897</v>
+        <v>10000000</v>
       </c>
       <c r="O58" t="n">
         <v>5000000</v>
       </c>
       <c r="P58" t="n">
-        <v>9916807</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="59">
@@ -3627,7 +3627,7 @@
         <v>5414146</v>
       </c>
       <c r="P59" t="n">
-        <v>11090757</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="60">
@@ -3678,10 +3678,10 @@
         <v>15927732</v>
       </c>
       <c r="O60" t="n">
-        <v>1015967</v>
+        <v>5000000</v>
       </c>
       <c r="P60" t="n">
-        <v>8664328</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="61">
@@ -3732,10 +3732,10 @@
         <v>32922101</v>
       </c>
       <c r="O61" t="n">
-        <v>4668348</v>
+        <v>5000000</v>
       </c>
       <c r="P61" t="n">
-        <v>14770589</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="62">
@@ -3789,7 +3789,7 @@
         <v>5000000</v>
       </c>
       <c r="P62" t="n">
-        <v>15802522</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="63">
@@ -3843,7 +3843,7 @@
         <v>9348740</v>
       </c>
       <c r="P63" t="n">
-        <v>14950141</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="64">
@@ -3894,7 +3894,7 @@
         <v>12234454</v>
       </c>
       <c r="O64" t="n">
-        <v>3790477</v>
+        <v>5000000</v>
       </c>
       <c r="P64" t="n">
         <v>101639856</v>
@@ -3948,10 +3948,10 @@
         <v>11817928</v>
       </c>
       <c r="O65" t="n">
-        <v>4192718</v>
+        <v>5000000</v>
       </c>
       <c r="P65" t="n">
-        <v>12756023</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="66">
@@ -4002,7 +4002,7 @@
         <v>41474230</v>
       </c>
       <c r="O66" t="n">
-        <v>3987676</v>
+        <v>5000000</v>
       </c>
       <c r="P66" t="n">
         <v>101639856</v>
@@ -4056,7 +4056,7 @@
         <v>61380113</v>
       </c>
       <c r="O67" t="n">
-        <v>4142578</v>
+        <v>5000000</v>
       </c>
       <c r="P67" t="n">
         <v>101639856</v>
@@ -4113,7 +4113,7 @@
         <v>8728852</v>
       </c>
       <c r="P68" t="n">
-        <v>11113166</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="69">
@@ -4215,13 +4215,13 @@
         <v>16499159</v>
       </c>
       <c r="N70" t="n">
-        <v>1726611</v>
+        <v>10000000</v>
       </c>
       <c r="O70" t="n">
-        <v>3664426</v>
+        <v>5000000</v>
       </c>
       <c r="P70" t="n">
-        <v>9389636</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="71">
@@ -4269,13 +4269,13 @@
         <v>17263025</v>
       </c>
       <c r="N71" t="n">
-        <v>16477469</v>
+        <v>12407732</v>
       </c>
       <c r="O71" t="n">
-        <v>2159024</v>
+        <v>5000000</v>
       </c>
       <c r="P71" t="n">
-        <v>26747275</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="72">
@@ -4323,13 +4323,13 @@
         <v>3596638</v>
       </c>
       <c r="N72" t="n">
-        <v>1842834</v>
+        <v>10000000</v>
       </c>
       <c r="O72" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P72" t="n">
-        <v>8511477</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="73">
@@ -4377,13 +4377,13 @@
         <v>9347899</v>
       </c>
       <c r="N73" t="n">
-        <v>1297870</v>
+        <v>10000000</v>
       </c>
       <c r="O73" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P73" t="n">
-        <v>12808155</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="74">
@@ -4431,13 +4431,13 @@
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>3880216</v>
+        <v>10000000</v>
       </c>
       <c r="O74" t="n">
-        <v>332000</v>
+        <v>5000000</v>
       </c>
       <c r="P74" t="n">
-        <v>5586157</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="75">
@@ -4485,13 +4485,13 @@
         <v>26086571</v>
       </c>
       <c r="N75" t="n">
-        <v>20939191</v>
+        <v>15767463</v>
       </c>
       <c r="O75" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P75" t="n">
-        <v>38488707</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="76">
@@ -4539,13 +4539,13 @@
         <v>4843697</v>
       </c>
       <c r="N76" t="n">
-        <v>12855562</v>
+        <v>10000000</v>
       </c>
       <c r="O76" t="n">
-        <v>2808144</v>
+        <v>5000000</v>
       </c>
       <c r="P76" t="n">
-        <v>16251265</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="77">
@@ -4593,13 +4593,13 @@
         <v>7099521</v>
       </c>
       <c r="N77" t="n">
-        <v>3712078</v>
+        <v>10000000</v>
       </c>
       <c r="O77" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P77" t="n">
-        <v>5974672</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="78">
@@ -4647,13 +4647,13 @@
         <v>5048739</v>
       </c>
       <c r="N78" t="n">
-        <v>5563093</v>
+        <v>10000000</v>
       </c>
       <c r="O78" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P78" t="n">
-        <v>9549326</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="79">
@@ -4701,13 +4701,13 @@
         <v>12413789</v>
       </c>
       <c r="N79" t="n">
-        <v>3046217</v>
+        <v>10000000</v>
       </c>
       <c r="O79" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P79" t="n">
-        <v>18779015</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="80">
@@ -4755,13 +4755,13 @@
         <v>3871428</v>
       </c>
       <c r="N80" t="n">
-        <v>26308909</v>
+        <v>19810925</v>
       </c>
       <c r="O80" t="n">
-        <v>928113</v>
+        <v>5000000</v>
       </c>
       <c r="P80" t="n">
-        <v>12238563</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="81">
@@ -4809,13 +4809,13 @@
         <v>15131983</v>
       </c>
       <c r="N81" t="n">
-        <v>12236566</v>
+        <v>10000000</v>
       </c>
       <c r="O81" t="n">
-        <v>849623</v>
+        <v>5000000</v>
       </c>
       <c r="P81" t="n">
-        <v>20505117</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="82">
@@ -4863,13 +4863,13 @@
         <v>3726890</v>
       </c>
       <c r="N82" t="n">
-        <v>14337989</v>
+        <v>10796678</v>
       </c>
       <c r="O82" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P82" t="n">
-        <v>13424333</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="83">
@@ -4917,13 +4917,13 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>8283448</v>
+        <v>10000000</v>
       </c>
       <c r="O83" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P83" t="n">
-        <v>8532176</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="84">
@@ -4971,13 +4971,13 @@
         <v>19946218</v>
       </c>
       <c r="N84" t="n">
-        <v>12939631</v>
+        <v>10000000</v>
       </c>
       <c r="O84" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P84" t="n">
-        <v>23289377</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="85">
@@ -5025,13 +5025,13 @@
         <v>4537815</v>
       </c>
       <c r="N85" t="n">
-        <v>14869881</v>
+        <v>11197199</v>
       </c>
       <c r="O85" t="n">
-        <v>2007841</v>
+        <v>5000000</v>
       </c>
       <c r="P85" t="n">
-        <v>14960442</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="86">
@@ -5079,13 +5079,13 @@
         <v>998000</v>
       </c>
       <c r="N86" t="n">
-        <v>8072113</v>
+        <v>10000000</v>
       </c>
       <c r="O86" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P86" t="n">
-        <v>3076208</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="87">
@@ -5133,13 +5133,13 @@
         <v>0</v>
       </c>
       <c r="N87" t="n">
-        <v>22422768</v>
+        <v>16884614</v>
       </c>
       <c r="O87" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P87" t="n">
-        <v>2420682</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="88">
@@ -5187,13 +5187,13 @@
         <v>3986554</v>
       </c>
       <c r="N88" t="n">
-        <v>15684909</v>
+        <v>11810925</v>
       </c>
       <c r="O88" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P88" t="n">
-        <v>13059356</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="89">
@@ -5241,13 +5241,13 @@
         <v>9694117</v>
       </c>
       <c r="N89" t="n">
-        <v>1571654</v>
+        <v>10000000</v>
       </c>
       <c r="O89" t="n">
-        <v>585140</v>
+        <v>5000000</v>
       </c>
       <c r="P89" t="n">
-        <v>15578892</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="90">
@@ -5295,13 +5295,13 @@
         <v>4467226</v>
       </c>
       <c r="N90" t="n">
-        <v>13920565</v>
+        <v>10482353</v>
       </c>
       <c r="O90" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P90" t="n">
-        <v>10175941</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="91">
@@ -5349,13 +5349,13 @@
         <v>12706537</v>
       </c>
       <c r="N91" t="n">
-        <v>1652747</v>
+        <v>10000000</v>
       </c>
       <c r="O91" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P91" t="n">
-        <v>10383076</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="92">
@@ -5403,13 +5403,13 @@
         <v>17110924</v>
       </c>
       <c r="N92" t="n">
-        <v>4385005</v>
+        <v>10000000</v>
       </c>
       <c r="O92" t="n">
-        <v>895378</v>
+        <v>5000000</v>
       </c>
       <c r="P92" t="n">
-        <v>19886150</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="93">
@@ -5457,13 +5457,13 @@
         <v>21316806</v>
       </c>
       <c r="N93" t="n">
-        <v>24953806</v>
+        <v>18790516</v>
       </c>
       <c r="O93" t="n">
-        <v>6640000</v>
+        <v>5000000</v>
       </c>
       <c r="P93" t="n">
-        <v>25366089</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="94">
@@ -5511,13 +5511,13 @@
         <v>4710084</v>
       </c>
       <c r="N94" t="n">
-        <v>9373747</v>
+        <v>10000000</v>
       </c>
       <c r="O94" t="n">
-        <v>2021016</v>
+        <v>5000000</v>
       </c>
       <c r="P94" t="n">
-        <v>11897988</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="95">
@@ -5568,7 +5568,7 @@
         <v>18199944</v>
       </c>
       <c r="O95" t="n">
-        <v>2288516</v>
+        <v>5000000</v>
       </c>
       <c r="P95" t="n">
         <v>101639856</v>
@@ -5676,10 +5676,10 @@
         <v>38117687</v>
       </c>
       <c r="O97" t="n">
-        <v>2792437</v>
+        <v>5000000</v>
       </c>
       <c r="P97" t="n">
-        <v>29056101</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="98">
@@ -5727,13 +5727,13 @@
         <v>5009243</v>
       </c>
       <c r="N98" t="n">
-        <v>6881393</v>
+        <v>10000000</v>
       </c>
       <c r="O98" t="n">
-        <v>2579832</v>
+        <v>5000000</v>
       </c>
       <c r="P98" t="n">
-        <v>1669748</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="99">
@@ -5838,10 +5838,10 @@
         <v>32118073</v>
       </c>
       <c r="O100" t="n">
-        <v>2322157</v>
+        <v>5000000</v>
       </c>
       <c r="P100" t="n">
-        <v>7489020</v>
+        <v>101639856</v>
       </c>
     </row>
     <row r="101">

</xml_diff>

<commit_message>
output: presupuestos_asesores_mayo_v3 - min_finans=16M
</commit_message>
<xml_diff>
--- a/docs/outputs/presupuestos_asesores_mayo.xlsx
+++ b/docs/outputs/presupuestos_asesores_mayo.xlsx
@@ -543,13 +543,13 @@
         <v>8411764</v>
       </c>
       <c r="N2" t="n">
-        <v>36378712</v>
+        <v>44563923</v>
       </c>
       <c r="O2" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P2" t="n">
-        <v>101639856</v>
+        <v>30878202</v>
       </c>
     </row>
     <row r="3">
@@ -597,13 +597,13 @@
         <v>7776470</v>
       </c>
       <c r="N3" t="n">
-        <v>10000000</v>
+        <v>12250000</v>
       </c>
       <c r="O3" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P3" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="4">
@@ -651,13 +651,13 @@
         <v>23529411</v>
       </c>
       <c r="N4" t="n">
-        <v>10000000</v>
+        <v>12250000</v>
       </c>
       <c r="O4" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P4" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="5">
@@ -705,13 +705,13 @@
         <v>22263865</v>
       </c>
       <c r="N5" t="n">
-        <v>23933054</v>
+        <v>29317992</v>
       </c>
       <c r="O5" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P5" t="n">
-        <v>101639856</v>
+        <v>26243825</v>
       </c>
     </row>
     <row r="6">
@@ -759,13 +759,13 @@
         <v>5642016</v>
       </c>
       <c r="N6" t="n">
-        <v>120946499</v>
+        <v>148159462</v>
       </c>
       <c r="O6" t="n">
-        <v>12807283</v>
+        <v>15688922</v>
       </c>
       <c r="P6" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="7">
@@ -813,13 +813,13 @@
         <v>4967226</v>
       </c>
       <c r="N7" t="n">
-        <v>44245659</v>
+        <v>54200933</v>
       </c>
       <c r="O7" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P7" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="8">
@@ -867,13 +867,13 @@
         <v>10627731</v>
       </c>
       <c r="N8" t="n">
-        <v>10000000</v>
+        <v>12250000</v>
       </c>
       <c r="O8" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P8" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="9">
@@ -921,13 +921,13 @@
         <v>14064705</v>
       </c>
       <c r="N9" t="n">
-        <v>53322970</v>
+        <v>65320639</v>
       </c>
       <c r="O9" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P9" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="10">
@@ -975,13 +975,13 @@
         <v>17435294</v>
       </c>
       <c r="N10" t="n">
-        <v>14825211</v>
+        <v>18160884</v>
       </c>
       <c r="O10" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P10" t="n">
-        <v>101639856</v>
+        <v>35659339</v>
       </c>
     </row>
     <row r="11">
@@ -1029,13 +1029,13 @@
         <v>41681546</v>
       </c>
       <c r="N11" t="n">
-        <v>62384539</v>
+        <v>76421061</v>
       </c>
       <c r="O11" t="n">
-        <v>5872550</v>
+        <v>7193874</v>
       </c>
       <c r="P11" t="n">
-        <v>101639856</v>
+        <v>55325407</v>
       </c>
     </row>
     <row r="12">
@@ -1083,13 +1083,13 @@
         <v>43616806</v>
       </c>
       <c r="N12" t="n">
-        <v>76396919</v>
+        <v>93586226</v>
       </c>
       <c r="O12" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P12" t="n">
-        <v>101639856</v>
+        <v>56568717</v>
       </c>
     </row>
     <row r="13">
@@ -1137,13 +1137,13 @@
         <v>14152100</v>
       </c>
       <c r="N13" t="n">
-        <v>31263866</v>
+        <v>38298236</v>
       </c>
       <c r="O13" t="n">
-        <v>5000000</v>
+        <v>6125000</v>
       </c>
       <c r="P13" t="n">
-        <v>101639856</v>
+        <v>19600000</v>
       </c>
     </row>
     <row r="14">
@@ -1197,7 +1197,7 @@
         <v>5000000</v>
       </c>
       <c r="P14" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="15">
@@ -1251,7 +1251,7 @@
         <v>5000000</v>
       </c>
       <c r="P15" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="16">
@@ -1305,7 +1305,7 @@
         <v>5000000</v>
       </c>
       <c r="P16" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="17">
@@ -1359,7 +1359,7 @@
         <v>5000000</v>
       </c>
       <c r="P17" t="n">
-        <v>101639856</v>
+        <v>22944314</v>
       </c>
     </row>
     <row r="18">
@@ -1413,7 +1413,7 @@
         <v>5000000</v>
       </c>
       <c r="P18" t="n">
-        <v>101639856</v>
+        <v>23027421</v>
       </c>
     </row>
     <row r="19">
@@ -1467,7 +1467,7 @@
         <v>5000000</v>
       </c>
       <c r="P19" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="20">
@@ -1521,7 +1521,7 @@
         <v>5000000</v>
       </c>
       <c r="P20" t="n">
-        <v>101639856</v>
+        <v>29705323</v>
       </c>
     </row>
     <row r="21">
@@ -1575,7 +1575,7 @@
         <v>5000000</v>
       </c>
       <c r="P21" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="22">
@@ -1629,7 +1629,7 @@
         <v>5000000</v>
       </c>
       <c r="P22" t="n">
-        <v>101639856</v>
+        <v>24211765</v>
       </c>
     </row>
     <row r="23">
@@ -1683,7 +1683,7 @@
         <v>5000000</v>
       </c>
       <c r="P23" t="n">
-        <v>101639856</v>
+        <v>25435015</v>
       </c>
     </row>
     <row r="24">
@@ -1737,7 +1737,7 @@
         <v>5000000</v>
       </c>
       <c r="P24" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="25">
@@ -1791,7 +1791,7 @@
         <v>8461132</v>
       </c>
       <c r="P25" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="26">
@@ -1845,7 +1845,7 @@
         <v>5000000</v>
       </c>
       <c r="P26" t="n">
-        <v>101639856</v>
+        <v>16629922</v>
       </c>
     </row>
     <row r="27">
@@ -1899,7 +1899,7 @@
         <v>5000000</v>
       </c>
       <c r="P27" t="n">
-        <v>101639856</v>
+        <v>24203244</v>
       </c>
     </row>
     <row r="28">
@@ -1953,7 +1953,7 @@
         <v>5000000</v>
       </c>
       <c r="P28" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="29">
@@ -2007,7 +2007,7 @@
         <v>7015687</v>
       </c>
       <c r="P29" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="30">
@@ -2061,7 +2061,7 @@
         <v>5000000</v>
       </c>
       <c r="P30" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="31">
@@ -2115,7 +2115,7 @@
         <v>18482606</v>
       </c>
       <c r="P31" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="32">
@@ -2169,7 +2169,7 @@
         <v>5000000</v>
       </c>
       <c r="P32" t="n">
-        <v>101639856</v>
+        <v>19699160</v>
       </c>
     </row>
     <row r="33">
@@ -2223,7 +2223,7 @@
         <v>8631491</v>
       </c>
       <c r="P33" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="34">
@@ -2277,7 +2277,7 @@
         <v>5000000</v>
       </c>
       <c r="P34" t="n">
-        <v>101639856</v>
+        <v>19690757</v>
       </c>
     </row>
     <row r="35">
@@ -2331,7 +2331,7 @@
         <v>5000000</v>
       </c>
       <c r="P35" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="36">
@@ -2385,7 +2385,7 @@
         <v>21088740</v>
       </c>
       <c r="P36" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="37">
@@ -2439,7 +2439,7 @@
         <v>5000000</v>
       </c>
       <c r="P37" t="n">
-        <v>101639856</v>
+        <v>18621202</v>
       </c>
     </row>
     <row r="38">
@@ -2493,7 +2493,7 @@
         <v>5000000</v>
       </c>
       <c r="P38" t="n">
-        <v>101639856</v>
+        <v>25875339</v>
       </c>
     </row>
     <row r="39">
@@ -2547,7 +2547,7 @@
         <v>5000000</v>
       </c>
       <c r="P39" t="n">
-        <v>101639856</v>
+        <v>16977031</v>
       </c>
     </row>
     <row r="40">
@@ -2601,7 +2601,7 @@
         <v>5000000</v>
       </c>
       <c r="P40" t="n">
-        <v>101639856</v>
+        <v>24900169</v>
       </c>
     </row>
     <row r="41">
@@ -2655,7 +2655,7 @@
         <v>5000000</v>
       </c>
       <c r="P41" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="42">
@@ -2703,13 +2703,13 @@
         <v>4010924</v>
       </c>
       <c r="N42" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O42" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P42" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="43">
@@ -2757,13 +2757,13 @@
         <v>8773109</v>
       </c>
       <c r="N43" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O43" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P43" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="44">
@@ -2811,13 +2811,13 @@
         <v>6868907</v>
       </c>
       <c r="N44" t="n">
-        <v>28027451</v>
+        <v>29008412</v>
       </c>
       <c r="O44" t="n">
-        <v>10158544</v>
+        <v>10514094</v>
       </c>
       <c r="P44" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="45">
@@ -2865,13 +2865,13 @@
         <v>20982352</v>
       </c>
       <c r="N45" t="n">
-        <v>24857984</v>
+        <v>25728014</v>
       </c>
       <c r="O45" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P45" t="n">
-        <v>101639856</v>
+        <v>17930144</v>
       </c>
     </row>
     <row r="46">
@@ -2919,13 +2919,13 @@
         <v>5103361</v>
       </c>
       <c r="N46" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O46" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P46" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="47">
@@ -2973,13 +2973,13 @@
         <v>24199999</v>
       </c>
       <c r="N47" t="n">
-        <v>17480566</v>
+        <v>18092386</v>
       </c>
       <c r="O47" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P47" t="n">
-        <v>101639856</v>
+        <v>29475284</v>
       </c>
     </row>
     <row r="48">
@@ -3027,13 +3027,13 @@
         <v>30847731</v>
       </c>
       <c r="N48" t="n">
-        <v>54062922</v>
+        <v>55955125</v>
       </c>
       <c r="O48" t="n">
-        <v>14968902</v>
+        <v>15492814</v>
       </c>
       <c r="P48" t="n">
-        <v>101639856</v>
+        <v>26601351</v>
       </c>
     </row>
     <row r="49">
@@ -3081,13 +3081,13 @@
         <v>7328571</v>
       </c>
       <c r="N49" t="n">
-        <v>39812325</v>
+        <v>41205757</v>
       </c>
       <c r="O49" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P49" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="50">
@@ -3135,13 +3135,13 @@
         <v>6914285</v>
       </c>
       <c r="N50" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O50" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P50" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="51">
@@ -3189,13 +3189,13 @@
         <v>25538655</v>
       </c>
       <c r="N51" t="n">
-        <v>47861625</v>
+        <v>49536782</v>
       </c>
       <c r="O51" t="n">
-        <v>9847536</v>
+        <v>10192200</v>
       </c>
       <c r="P51" t="n">
-        <v>101639856</v>
+        <v>20844814</v>
       </c>
     </row>
     <row r="52">
@@ -3243,13 +3243,13 @@
         <v>2079831</v>
       </c>
       <c r="N52" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O52" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P52" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="53">
@@ -3297,13 +3297,13 @@
         <v>16697478</v>
       </c>
       <c r="N53" t="n">
-        <v>43523530</v>
+        <v>45046854</v>
       </c>
       <c r="O53" t="n">
-        <v>7048460</v>
+        <v>7295157</v>
       </c>
       <c r="P53" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="54">
@@ -3351,13 +3351,13 @@
         <v>14551680</v>
       </c>
       <c r="N54" t="n">
-        <v>10000000</v>
+        <v>10350000</v>
       </c>
       <c r="O54" t="n">
-        <v>5000000</v>
+        <v>5175000</v>
       </c>
       <c r="P54" t="n">
-        <v>101639856</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="55">
@@ -3405,13 +3405,13 @@
         <v>20524033</v>
       </c>
       <c r="N55" t="n">
-        <v>77352468</v>
+        <v>80059805</v>
       </c>
       <c r="O55" t="n">
-        <v>5033054</v>
+        <v>5209211</v>
       </c>
       <c r="P55" t="n">
-        <v>101639856</v>
+        <v>24725448</v>
       </c>
     </row>
     <row r="56">
@@ -3459,13 +3459,13 @@
         <v>31865546</v>
       </c>
       <c r="N56" t="n">
-        <v>10000000</v>
+        <v>11020000</v>
       </c>
       <c r="O56" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P56" t="n">
-        <v>101639856</v>
+        <v>32031159</v>
       </c>
     </row>
     <row r="57">
@@ -3513,13 +3513,13 @@
         <v>24813067</v>
       </c>
       <c r="N57" t="n">
-        <v>15572269</v>
+        <v>17160641</v>
       </c>
       <c r="O57" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P57" t="n">
-        <v>101639856</v>
+        <v>20574774</v>
       </c>
     </row>
     <row r="58">
@@ -3567,13 +3567,13 @@
         <v>12105042</v>
       </c>
       <c r="N58" t="n">
-        <v>10000000</v>
+        <v>11020000</v>
       </c>
       <c r="O58" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P58" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="59">
@@ -3621,13 +3621,13 @@
         <v>18513445</v>
       </c>
       <c r="N59" t="n">
-        <v>23738656</v>
+        <v>26159999</v>
       </c>
       <c r="O59" t="n">
-        <v>5414146</v>
+        <v>5966389</v>
       </c>
       <c r="P59" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="60">
@@ -3675,13 +3675,13 @@
         <v>6827731</v>
       </c>
       <c r="N60" t="n">
-        <v>15927732</v>
+        <v>17552361</v>
       </c>
       <c r="O60" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P60" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="61">
@@ -3729,13 +3729,13 @@
         <v>18628571</v>
       </c>
       <c r="N61" t="n">
-        <v>32922101</v>
+        <v>36280156</v>
       </c>
       <c r="O61" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P61" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="62">
@@ -3783,13 +3783,13 @@
         <v>14882352</v>
       </c>
       <c r="N62" t="n">
-        <v>12960785</v>
+        <v>14282786</v>
       </c>
       <c r="O62" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P62" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="63">
@@ -3837,13 +3837,13 @@
         <v>18955462</v>
       </c>
       <c r="N63" t="n">
-        <v>22600281</v>
+        <v>24905510</v>
       </c>
       <c r="O63" t="n">
-        <v>9348740</v>
+        <v>10302312</v>
       </c>
       <c r="P63" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="64">
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>12234454</v>
+        <v>13482369</v>
       </c>
       <c r="O64" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P64" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="65">
@@ -3945,13 +3945,13 @@
         <v>19705042</v>
       </c>
       <c r="N65" t="n">
-        <v>11817928</v>
+        <v>13023357</v>
       </c>
       <c r="O65" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P65" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="66">
@@ -3999,13 +3999,13 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>41474230</v>
+        <v>45704602</v>
       </c>
       <c r="O66" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P66" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="67">
@@ -4053,13 +4053,13 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>61380113</v>
+        <v>67640885</v>
       </c>
       <c r="O67" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P67" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="68">
@@ -4107,13 +4107,13 @@
         <v>19928571</v>
       </c>
       <c r="N68" t="n">
-        <v>23615547</v>
+        <v>26024333</v>
       </c>
       <c r="O68" t="n">
-        <v>8728852</v>
+        <v>9619195</v>
       </c>
       <c r="P68" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="69">
@@ -4161,13 +4161,13 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>10000000</v>
+        <v>11020000</v>
       </c>
       <c r="O69" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P69" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="70">
@@ -4215,13 +4215,13 @@
         <v>16499159</v>
       </c>
       <c r="N70" t="n">
-        <v>10000000</v>
+        <v>11020000</v>
       </c>
       <c r="O70" t="n">
-        <v>5000000</v>
+        <v>5510000</v>
       </c>
       <c r="P70" t="n">
-        <v>101639856</v>
+        <v>17632000</v>
       </c>
     </row>
     <row r="71">
@@ -4275,7 +4275,7 @@
         <v>5000000</v>
       </c>
       <c r="P71" t="n">
-        <v>101639856</v>
+        <v>20141020</v>
       </c>
     </row>
     <row r="72">
@@ -4329,7 +4329,7 @@
         <v>5000000</v>
       </c>
       <c r="P72" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="73">
@@ -4383,7 +4383,7 @@
         <v>5000000</v>
       </c>
       <c r="P73" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="74">
@@ -4437,7 +4437,7 @@
         <v>5000000</v>
       </c>
       <c r="P74" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="75">
@@ -4491,7 +4491,7 @@
         <v>5000000</v>
       </c>
       <c r="P75" t="n">
-        <v>101639856</v>
+        <v>28982460</v>
       </c>
     </row>
     <row r="76">
@@ -4545,7 +4545,7 @@
         <v>5000000</v>
       </c>
       <c r="P76" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="77">
@@ -4599,7 +4599,7 @@
         <v>5000000</v>
       </c>
       <c r="P77" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="78">
@@ -4653,7 +4653,7 @@
         <v>5000000</v>
       </c>
       <c r="P78" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="79">
@@ -4707,7 +4707,7 @@
         <v>5000000</v>
       </c>
       <c r="P79" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="80">
@@ -4761,7 +4761,7 @@
         <v>5000000</v>
       </c>
       <c r="P80" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="81">
@@ -4815,7 +4815,7 @@
         <v>5000000</v>
       </c>
       <c r="P81" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="82">
@@ -4869,7 +4869,7 @@
         <v>5000000</v>
       </c>
       <c r="P82" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="83">
@@ -4923,7 +4923,7 @@
         <v>5000000</v>
       </c>
       <c r="P83" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="84">
@@ -4977,7 +4977,7 @@
         <v>5000000</v>
       </c>
       <c r="P84" t="n">
-        <v>101639856</v>
+        <v>17537181</v>
       </c>
     </row>
     <row r="85">
@@ -5031,7 +5031,7 @@
         <v>5000000</v>
       </c>
       <c r="P85" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="86">
@@ -5085,7 +5085,7 @@
         <v>5000000</v>
       </c>
       <c r="P86" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="87">
@@ -5139,7 +5139,7 @@
         <v>5000000</v>
       </c>
       <c r="P87" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="88">
@@ -5193,7 +5193,7 @@
         <v>5000000</v>
       </c>
       <c r="P88" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="89">
@@ -5247,7 +5247,7 @@
         <v>5000000</v>
       </c>
       <c r="P89" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="90">
@@ -5301,7 +5301,7 @@
         <v>5000000</v>
       </c>
       <c r="P90" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="91">
@@ -5355,7 +5355,7 @@
         <v>5000000</v>
       </c>
       <c r="P91" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="92">
@@ -5409,7 +5409,7 @@
         <v>5000000</v>
       </c>
       <c r="P92" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="93">
@@ -5463,7 +5463,7 @@
         <v>5000000</v>
       </c>
       <c r="P93" t="n">
-        <v>101639856</v>
+        <v>19100970</v>
       </c>
     </row>
     <row r="94">
@@ -5517,7 +5517,7 @@
         <v>5000000</v>
       </c>
       <c r="P94" t="n">
-        <v>101639856</v>
+        <v>16000000</v>
       </c>
     </row>
     <row r="95">
@@ -5565,13 +5565,13 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>18199944</v>
+        <v>19255541</v>
       </c>
       <c r="O95" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P95" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
     <row r="96">
@@ -5619,13 +5619,13 @@
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>10000000</v>
+        <v>10580000</v>
       </c>
       <c r="O96" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P96" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
     <row r="97">
@@ -5673,13 +5673,13 @@
         <v>19716100</v>
       </c>
       <c r="N97" t="n">
-        <v>38117687</v>
+        <v>40328513</v>
       </c>
       <c r="O97" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P97" t="n">
-        <v>101639856</v>
+        <v>30741355</v>
       </c>
     </row>
     <row r="98">
@@ -5727,13 +5727,13 @@
         <v>5009243</v>
       </c>
       <c r="N98" t="n">
-        <v>10000000</v>
+        <v>10580000</v>
       </c>
       <c r="O98" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P98" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
     <row r="99">
@@ -5781,13 +5781,13 @@
         <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>10000000</v>
+        <v>10580000</v>
       </c>
       <c r="O99" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P99" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
     <row r="100">
@@ -5835,13 +5835,13 @@
         <v>1050420</v>
       </c>
       <c r="N100" t="n">
-        <v>32118073</v>
+        <v>33980922</v>
       </c>
       <c r="O100" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P100" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
     <row r="101">
@@ -5889,13 +5889,13 @@
         <v>0</v>
       </c>
       <c r="N101" t="n">
-        <v>10000000</v>
+        <v>10580000</v>
       </c>
       <c r="O101" t="n">
-        <v>5000000</v>
+        <v>5290000</v>
       </c>
       <c r="P101" t="n">
-        <v>101639856</v>
+        <v>16928000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>